<commit_message>
Daily oil & gas forecast 2026-10-12
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -1140,7 +1140,7 @@
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
-        <v>-0.0768228727027699</v>
+        <v>-0.076822872702769</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>2.52021483771038</v>
@@ -1152,7 +1152,7 @@
         <v>2.35227328376466</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.51295988955555</v>
+        <v>3.51295988955556</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>0.219653179190751</v>

</xml_diff>

<commit_message>
Daily oil & gas forecast 2026-10-13
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -1140,7 +1140,7 @@
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
-        <v>-0.076822872702769</v>
+        <v>-0.0768228727027699</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>2.52021483771038</v>
@@ -1152,7 +1152,7 @@
         <v>2.35227328376466</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.51295988955556</v>
+        <v>3.51295988955555</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>0.219653179190751</v>

</xml_diff>

<commit_message>
Daily oil & gas forecast 2026-10-14
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -692,7 +692,7 @@
       </c>
       <c r="J18" s="5" t="n">
         <f aca="false">Details!G7</f>
-        <v>2.79722669571061</v>
+        <v>2.82654098517657</v>
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Details!O7</f>
@@ -1136,26 +1136,26 @@
         <v>3.03</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>2.79722669571061</v>
+        <v>2.82654098517657</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
-        <v>-0.0768228727027699</v>
+        <v>-0.0671481897107039</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>2.52021483771038</v>
+        <v>2.54662610690867</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>3.19134968337202</v>
+        <v>3.22479429068573</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2.35227328376466</v>
+        <v>2.37692456428084</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.51295988955555</v>
+        <v>3.54977489752136</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0.219653179190751</v>
+        <v>0.246146435452794</v>
       </c>
       <c r="N7" s="14" t="n">
         <v>0.140745706717376</v>

</xml_diff>

<commit_message>
Daily oil & gas forecast 2026-10-15
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -1140,7 +1140,7 @@
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
-        <v>-0.0671481897107039</v>
+        <v>-0.0671481897107029</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>2.54662610690867</v>
@@ -1149,7 +1149,7 @@
         <v>3.22479429068573</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2.37692456428084</v>
+        <v>2.37692456428085</v>
       </c>
       <c r="L7" s="11" t="n">
         <v>3.54977489752136</v>

</xml_diff>

<commit_message>
Daily oil & gas forecast 2026-10-16
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Henry Hub ($/MMBtu)</t>
   </si>
   <si>
-    <t xml:space="preserve">Forecast made on prices up to 2026-10-06; 7 day = 2026-10-13, 15 day = 2026-10-21.</t>
+    <t xml:space="preserve">Forecast made on prices up to 2026-10-14; 7 day = 2026-10-21, 15 day = 2026-10-29.</t>
   </si>
   <si>
     <t xml:space="preserve">Prices in $/bbl except Henry Hub ($/MMBtu).</t>
@@ -642,19 +642,19 @@
       </c>
       <c r="H16" s="5" t="n">
         <f aca="false">Details!G2</f>
-        <v>125.44</v>
+        <v>126.55</v>
       </c>
       <c r="I16" s="6" t="n">
         <f aca="false">Details!O2</f>
-        <v>0.953690891374132</v>
+        <v>0.953656995159445</v>
       </c>
       <c r="J16" s="5" t="n">
         <f aca="false">Details!G3</f>
-        <v>125.44</v>
+        <v>126.55</v>
       </c>
       <c r="K16" s="6" t="n">
         <f aca="false">Details!O3</f>
-        <v>0.931231617303026</v>
+        <v>0.931187057374352</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -663,19 +663,19 @@
       </c>
       <c r="H17" s="5" t="n">
         <f aca="false">Details!G4</f>
-        <v>96.24</v>
+        <v>101.91</v>
       </c>
       <c r="I17" s="6" t="n">
         <f aca="false">Details!O4</f>
-        <v>0.953911226105119</v>
+        <v>0.953936744788498</v>
       </c>
       <c r="J17" s="5" t="n">
         <f aca="false">Details!G5</f>
-        <v>96.24</v>
+        <v>101.91</v>
       </c>
       <c r="K17" s="6" t="n">
         <f aca="false">Details!O5</f>
-        <v>0.931415532709249</v>
+        <v>0.931518911250012</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -684,19 +684,19 @@
       </c>
       <c r="H18" s="5" t="n">
         <f aca="false">Details!G6</f>
-        <v>3.03</v>
+        <v>3.22</v>
       </c>
       <c r="I18" s="6" t="n">
         <f aca="false">Details!O6</f>
-        <v>0.890209800812561</v>
+        <v>0.890190177554327</v>
       </c>
       <c r="J18" s="5" t="n">
         <f aca="false">Details!G7</f>
-        <v>2.82654098517657</v>
+        <v>3.06796931770086</v>
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Details!O7</f>
-        <v>0.859254293282624</v>
+        <v>0.85915507269062</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -822,51 +822,51 @@
         <v>7</v>
       </c>
       <c r="D2" s="10" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="E2" s="10" t="n">
-        <v>46308</v>
+        <v>46316</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>125.44</v>
+        <v>126.55</v>
       </c>
       <c r="G2" s="11" t="n">
-        <v>125.44</v>
+        <v>126.55</v>
       </c>
       <c r="H2" s="12" t="n">
         <f aca="false">G2/F2-1</f>
         <v>0</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>106.291463394673</v>
+        <v>110.248766328426</v>
       </c>
       <c r="J2" s="11" t="n">
-        <v>146.555044434495</v>
+        <v>144.167048766318</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>93.6750738927436</v>
+        <v>99.1272472220683</v>
       </c>
       <c r="L2" s="11" t="n">
-        <v>160.560213427967</v>
+        <v>155.578630189186</v>
       </c>
       <c r="M2" s="13" t="n">
-        <v>0.53073967339097</v>
+        <v>0.532885261641863</v>
       </c>
       <c r="N2" s="14" t="n">
-        <v>0.0463091086258684</v>
+        <v>0.0463430048405547</v>
       </c>
       <c r="O2" s="15" t="n">
         <f aca="false">1-N2</f>
-        <v>0.953690891374132</v>
+        <v>0.953656995159445</v>
       </c>
       <c r="P2" s="13" t="n">
-        <v>0.693563880883766</v>
+        <v>0.693230916946712</v>
       </c>
       <c r="Q2" s="13" t="n">
-        <v>0.78544061302682</v>
+        <v>0.783369803063457</v>
       </c>
       <c r="R2" s="13" t="n">
-        <v>0.79110251450677</v>
+        <v>0.78957528957529</v>
       </c>
       <c r="S2" s="16" t="s">
         <v>31</v>
@@ -883,51 +883,51 @@
         <v>15</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>46316</v>
+        <v>46324</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>125.44</v>
+        <v>126.55</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>125.44</v>
+        <v>126.55</v>
       </c>
       <c r="H3" s="12" t="n">
         <f aca="false">G3/F3-1</f>
         <v>0</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>97.0936649645044</v>
+        <v>102.258710223637</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>158.187218141549</v>
+        <v>153.647994666834</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>79.3246556537947</v>
+        <v>86.2471785454344</v>
       </c>
       <c r="L3" s="11" t="n">
-        <v>187.375085641985</v>
+        <v>177.034573514863</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>0.549614643545279</v>
+        <v>0.552238805970149</v>
       </c>
       <c r="N3" s="14" t="n">
-        <v>0.068768382696974</v>
+        <v>0.0688129426256479</v>
       </c>
       <c r="O3" s="15" t="n">
         <f aca="false">1-N3</f>
-        <v>0.931231617303026</v>
+        <v>0.931187057374352</v>
       </c>
       <c r="P3" s="13" t="n">
-        <v>0.533236994219653</v>
+        <v>0.532980259990371</v>
       </c>
       <c r="Q3" s="13" t="n">
-        <v>0.796143250688705</v>
+        <v>0.79295154185022</v>
       </c>
       <c r="R3" s="13" t="n">
-        <v>0.782778864970646</v>
+        <v>0.783203125</v>
       </c>
       <c r="S3" s="16" t="s">
         <v>31</v>
@@ -944,51 +944,51 @@
         <v>7</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>46308</v>
+        <v>46316</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>96.24</v>
+        <v>101.91</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>96.24</v>
+        <v>101.91</v>
       </c>
       <c r="H4" s="12" t="n">
         <f aca="false">G4/F4-1</f>
         <v>0</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>83.6557998104468</v>
+        <v>90.6080288047093</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>109.280147786715</v>
+        <v>113.38424731664</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>75.0444002198064</v>
+        <v>82.6947809002898</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>116.995208906954</v>
+        <v>120.071759093373</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>0.535542747358309</v>
+        <v>0.537205952952472</v>
       </c>
       <c r="N4" s="14" t="n">
-        <v>0.046088773894881</v>
+        <v>0.0460632552115024</v>
       </c>
       <c r="O4" s="15" t="n">
         <f aca="false">1-N4</f>
-        <v>0.953911226105119</v>
+        <v>0.953936744788498</v>
       </c>
       <c r="P4" s="13" t="n">
-        <v>0.699327569644573</v>
+        <v>0.699471915506481</v>
       </c>
       <c r="Q4" s="13" t="n">
-        <v>0.801860974274767</v>
+        <v>0.800875273522976</v>
       </c>
       <c r="R4" s="13" t="n">
-        <v>0.808510638297872</v>
+        <v>0.810810810810811</v>
       </c>
       <c r="S4" s="16" t="s">
         <v>31</v>
@@ -1005,51 +1005,51 @@
         <v>15</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>46316</v>
+        <v>46324</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>96.24</v>
+        <v>101.91</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>96.24</v>
+        <v>101.91</v>
       </c>
       <c r="H5" s="12" t="n">
         <f aca="false">G5/F5-1</f>
         <v>0</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>77.9361598488761</v>
+        <v>85.503157928385</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>115.463104849543</v>
+        <v>118.739817839881</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>65.7989979223051</v>
+        <v>74.0535193838932</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>130.661835448597</v>
+        <v>131.729115552947</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>0.554431599229287</v>
+        <v>0.556571978815599</v>
       </c>
       <c r="N5" s="14" t="n">
-        <v>0.0685844672907508</v>
+        <v>0.0684810887499878</v>
       </c>
       <c r="O5" s="15" t="n">
         <f aca="false">1-N5</f>
-        <v>0.931415532709249</v>
+        <v>0.931518911250012</v>
       </c>
       <c r="P5" s="13" t="n">
-        <v>0.533718689788054</v>
+        <v>0.535387578237843</v>
       </c>
       <c r="Q5" s="13" t="n">
-        <v>0.808815426997245</v>
+        <v>0.80726872246696</v>
       </c>
       <c r="R5" s="13" t="n">
-        <v>0.816046966731898</v>
+        <v>0.814453125</v>
       </c>
       <c r="S5" s="16" t="s">
         <v>31</v>
@@ -1066,51 +1066,51 @@
         <v>7</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>46308</v>
+        <v>46316</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>3.03</v>
+        <v>3.22</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>3.03</v>
+        <v>3.22</v>
       </c>
       <c r="H6" s="12" t="n">
         <f aca="false">G6/F6-1</f>
         <v>0</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>2.80160460799405</v>
+        <v>2.98515424817596</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>3.28261561527103</v>
+        <v>3.47907489430198</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>2.64892141449828</v>
+        <v>2.82781656416723</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>3.50465826646317</v>
+        <v>3.70623153650955</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>0.497118155619597</v>
+        <v>0.498799807969275</v>
       </c>
       <c r="N6" s="14" t="n">
-        <v>0.109790199187439</v>
+        <v>0.109809822445673</v>
       </c>
       <c r="O6" s="15" t="n">
         <f aca="false">1-N6</f>
-        <v>0.890209800812561</v>
+        <v>0.890190177554327</v>
       </c>
       <c r="P6" s="13" t="n">
-        <v>0.420749279538905</v>
+        <v>0.420067210753721</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>0.80952380952381</v>
+        <v>0.811269146608315</v>
       </c>
       <c r="R6" s="13" t="n">
-        <v>0.823984526112186</v>
+        <v>0.826254826254826</v>
       </c>
       <c r="S6" s="16" t="s">
         <v>31</v>
@@ -1127,51 +1127,51 @@
         <v>15</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>46316</v>
+        <v>46324</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>3.03</v>
+        <v>3.22</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>2.82654098517657</v>
+        <v>3.06796931770086</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
-        <v>-0.0671481897107029</v>
+        <v>-0.0472144976084287</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>2.54662610690867</v>
+        <v>2.77402613657568</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>3.22479429068573</v>
+        <v>3.4895117560625</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2.37692456428085</v>
+        <v>2.59412098267082</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.54977489752136</v>
+        <v>3.80845965740818</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0.246146435452794</v>
+        <v>0.321136254212807</v>
       </c>
       <c r="N7" s="14" t="n">
-        <v>0.140745706717376</v>
+        <v>0.14084492730938</v>
       </c>
       <c r="O7" s="15" t="n">
         <f aca="false">1-N7</f>
-        <v>0.859254293282624</v>
+        <v>0.85915507269062</v>
       </c>
       <c r="P7" s="13" t="n">
-        <v>0.276011560693642</v>
+        <v>0.271545498314877</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>0.809366391184573</v>
+        <v>0.810022026431718</v>
       </c>
       <c r="R7" s="13" t="n">
-        <v>0.841487279843444</v>
+        <v>0.841796875</v>
       </c>
       <c r="S7" s="16" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Daily oil & gas forecast 2026-10-20
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -692,7 +692,7 @@
       </c>
       <c r="J18" s="5" t="n">
         <f aca="false">Details!G7</f>
-        <v>3.06796931770086</v>
+        <v>3.10941090365116</v>
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Details!O7</f>
@@ -1136,26 +1136,26 @@
         <v>3.22</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>3.06796931770086</v>
+        <v>3.10941090365116</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
-        <v>-0.0472144976084287</v>
+        <v>-0.0343444398598879</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>2.77402613657568</v>
+        <v>2.81149719011719</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>3.4895117560625</v>
+        <v>3.53664746257987</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2.59412098267082</v>
+        <v>2.62916190926958</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.80845965740818</v>
+        <v>3.85990365566466</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0.321136254212807</v>
+        <v>0.37217140105922</v>
       </c>
       <c r="N7" s="14" t="n">
         <v>0.14084492730938</v>

</xml_diff>

<commit_message>
Daily oil & gas forecast 2026-10-22
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
   <si>
     <t xml:space="preserve">Crude oil Price forecast per bbl</t>
   </si>
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Henry Hub ($/MMBtu)</t>
   </si>
   <si>
-    <t xml:space="preserve">Forecast made on prices up to 2026-10-14; 7 day = 2026-10-21, 15 day = 2026-10-29.</t>
+    <t xml:space="preserve">Forecast made on prices up to 2026-10-20; 7 day = 2026-10-27, 15 day = 2026-11-04.</t>
   </si>
   <si>
     <t xml:space="preserve">Prices in $/bbl except Henry Hub ($/MMBtu).</t>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t xml:space="preserve">$/MMBtu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ridge regression</t>
   </si>
   <si>
     <t xml:space="preserve">Data: FRED / EIA APIs + EIA spot prices (github.com/datasets mirror). Blue = model output (python run_forecast.py); black = formula.</t>
@@ -642,19 +639,19 @@
       </c>
       <c r="H16" s="5" t="n">
         <f aca="false">Details!G2</f>
-        <v>126.55</v>
+        <v>115.22</v>
       </c>
       <c r="I16" s="6" t="n">
         <f aca="false">Details!O2</f>
-        <v>0.953656995159445</v>
+        <v>0.953555293492327</v>
       </c>
       <c r="J16" s="5" t="n">
         <f aca="false">Details!G3</f>
-        <v>126.55</v>
+        <v>115.22</v>
       </c>
       <c r="K16" s="6" t="n">
         <f aca="false">Details!O3</f>
-        <v>0.931187057374352</v>
+        <v>0.931226967224115</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -663,19 +660,19 @@
       </c>
       <c r="H17" s="5" t="n">
         <f aca="false">Details!G4</f>
-        <v>101.91</v>
+        <v>107.89</v>
       </c>
       <c r="I17" s="6" t="n">
         <f aca="false">Details!O4</f>
-        <v>0.953936744788498</v>
+        <v>0.953872727483083</v>
       </c>
       <c r="J17" s="5" t="n">
         <f aca="false">Details!G5</f>
-        <v>101.91</v>
+        <v>107.89</v>
       </c>
       <c r="K17" s="6" t="n">
         <f aca="false">Details!O5</f>
-        <v>0.931518911250012</v>
+        <v>0.931561064272199</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -684,19 +681,19 @@
       </c>
       <c r="H18" s="5" t="n">
         <f aca="false">Details!G6</f>
-        <v>3.22</v>
+        <v>3.1</v>
       </c>
       <c r="I18" s="6" t="n">
         <f aca="false">Details!O6</f>
-        <v>0.890190177554327</v>
+        <v>0.890135513243169</v>
       </c>
       <c r="J18" s="5" t="n">
         <f aca="false">Details!G7</f>
-        <v>3.10941090365116</v>
+        <v>3.1</v>
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Details!O7</f>
-        <v>0.85915507269062</v>
+        <v>0.846642277960824</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -822,51 +819,51 @@
         <v>7</v>
       </c>
       <c r="D2" s="10" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="E2" s="10" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>126.55</v>
+        <v>115.22</v>
       </c>
       <c r="G2" s="11" t="n">
-        <v>126.55</v>
+        <v>115.22</v>
       </c>
       <c r="H2" s="12" t="n">
         <f aca="false">G2/F2-1</f>
         <v>0</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>110.248766328426</v>
+        <v>101.308872623481</v>
       </c>
       <c r="J2" s="11" t="n">
-        <v>144.167048766318</v>
+        <v>130.171709702822</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>99.1272472220683</v>
+        <v>91.6669081069355</v>
       </c>
       <c r="L2" s="11" t="n">
-        <v>155.578630189186</v>
+        <v>139.792901681923</v>
       </c>
       <c r="M2" s="13" t="n">
-        <v>0.532885261641863</v>
+        <v>0.53314121037464</v>
       </c>
       <c r="N2" s="14" t="n">
-        <v>0.0463430048405547</v>
+        <v>0.046444706507673</v>
       </c>
       <c r="O2" s="15" t="n">
         <f aca="false">1-N2</f>
-        <v>0.953656995159445</v>
+        <v>0.953555293492327</v>
       </c>
       <c r="P2" s="13" t="n">
-        <v>0.693230916946712</v>
+        <v>0.69164265129683</v>
       </c>
       <c r="Q2" s="13" t="n">
-        <v>0.783369803063457</v>
+        <v>0.784345922276957</v>
       </c>
       <c r="R2" s="13" t="n">
-        <v>0.78957528957529</v>
+        <v>0.789168278529981</v>
       </c>
       <c r="S2" s="16" t="s">
         <v>31</v>
@@ -883,51 +880,51 @@
         <v>15</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>46324</v>
+        <v>46330</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>126.55</v>
+        <v>115.22</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>126.55</v>
+        <v>115.22</v>
       </c>
       <c r="H3" s="12" t="n">
         <f aca="false">G3/F3-1</f>
         <v>0</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>102.258710223637</v>
+        <v>94.8479044038997</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>153.647994666834</v>
+        <v>138.17221400397</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>86.2471785454344</v>
+        <v>80.7498111838232</v>
       </c>
       <c r="L3" s="11" t="n">
-        <v>177.034573514863</v>
+        <v>157.766705422609</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>0.552238805970149</v>
+        <v>0.553468208092486</v>
       </c>
       <c r="N3" s="14" t="n">
-        <v>0.0688129426256479</v>
+        <v>0.0687730327758854</v>
       </c>
       <c r="O3" s="15" t="n">
         <f aca="false">1-N3</f>
-        <v>0.931187057374352</v>
+        <v>0.931226967224115</v>
       </c>
       <c r="P3" s="13" t="n">
-        <v>0.532980259990371</v>
+        <v>0.533718689788054</v>
       </c>
       <c r="Q3" s="13" t="n">
-        <v>0.79295154185022</v>
+        <v>0.788980716253444</v>
       </c>
       <c r="R3" s="13" t="n">
-        <v>0.783203125</v>
+        <v>0.772994129158513</v>
       </c>
       <c r="S3" s="16" t="s">
         <v>31</v>
@@ -944,51 +941,51 @@
         <v>7</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>101.91</v>
+        <v>107.89</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>101.91</v>
+        <v>107.89</v>
       </c>
       <c r="H4" s="12" t="n">
         <f aca="false">G4/F4-1</f>
         <v>0</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>90.6080288047093</v>
+        <v>95.4250684796895</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>113.38424731664</v>
+        <v>120.70865748815</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>82.6947809002898</v>
+        <v>86.710635653351</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>120.071759093373</v>
+        <v>128.081793069465</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>0.537205952952472</v>
+        <v>0.538424591738713</v>
       </c>
       <c r="N4" s="14" t="n">
-        <v>0.0460632552115024</v>
+        <v>0.0461272725169175</v>
       </c>
       <c r="O4" s="15" t="n">
         <f aca="false">1-N4</f>
-        <v>0.953936744788498</v>
+        <v>0.953872727483083</v>
       </c>
       <c r="P4" s="13" t="n">
-        <v>0.699471915506481</v>
+        <v>0.698366954851105</v>
       </c>
       <c r="Q4" s="13" t="n">
-        <v>0.800875273522976</v>
+        <v>0.799671592775041</v>
       </c>
       <c r="R4" s="13" t="n">
-        <v>0.810810810810811</v>
+        <v>0.806576402321083</v>
       </c>
       <c r="S4" s="16" t="s">
         <v>31</v>
@@ -1005,51 +1002,51 @@
         <v>15</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>46324</v>
+        <v>46330</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>101.91</v>
+        <v>107.89</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>101.91</v>
+        <v>107.89</v>
       </c>
       <c r="H5" s="12" t="n">
         <f aca="false">G5/F5-1</f>
         <v>0</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>85.503157928385</v>
+        <v>90.2883445378342</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>118.739817839881</v>
+        <v>126.607148094806</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>74.0535193838932</v>
+        <v>77.2523905273769</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>131.729115552947</v>
+        <v>141.135917535299</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>0.556571978815599</v>
+        <v>0.558285163776493</v>
       </c>
       <c r="N5" s="14" t="n">
-        <v>0.0684810887499878</v>
+        <v>0.0684389357278012</v>
       </c>
       <c r="O5" s="15" t="n">
         <f aca="false">1-N5</f>
-        <v>0.931518911250012</v>
+        <v>0.931561064272199</v>
       </c>
       <c r="P5" s="13" t="n">
-        <v>0.535387578237843</v>
+        <v>0.536127167630058</v>
       </c>
       <c r="Q5" s="13" t="n">
-        <v>0.80726872246696</v>
+        <v>0.806060606060606</v>
       </c>
       <c r="R5" s="13" t="n">
-        <v>0.814453125</v>
+        <v>0.814090019569472</v>
       </c>
       <c r="S5" s="16" t="s">
         <v>31</v>
@@ -1066,51 +1063,51 @@
         <v>7</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>3.22</v>
+        <v>3.1</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>3.22</v>
+        <v>3.1</v>
       </c>
       <c r="H6" s="12" t="n">
         <f aca="false">G6/F6-1</f>
         <v>0</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>2.98515424817596</v>
+        <v>2.86517013121415</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>3.47907489430198</v>
+        <v>3.35983858732731</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>2.82781656416723</v>
+        <v>2.70824005693516</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>3.70623153650955</v>
+        <v>3.58831554209777</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>0.498799807969275</v>
+        <v>0.498559077809798</v>
       </c>
       <c r="N6" s="14" t="n">
-        <v>0.109809822445673</v>
+        <v>0.109864486756831</v>
       </c>
       <c r="O6" s="15" t="n">
         <f aca="false">1-N6</f>
-        <v>0.890190177554327</v>
+        <v>0.890135513243169</v>
       </c>
       <c r="P6" s="13" t="n">
-        <v>0.420067210753721</v>
+        <v>0.419308357348703</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>0.811269146608315</v>
+        <v>0.812807881773399</v>
       </c>
       <c r="R6" s="13" t="n">
-        <v>0.826254826254826</v>
+        <v>0.831721470019342</v>
       </c>
       <c r="S6" s="16" t="s">
         <v>31</v>
@@ -1127,74 +1124,74 @@
         <v>15</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>46324</v>
+        <v>46330</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>3.22</v>
+        <v>3.1</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>3.10941090365116</v>
+        <v>3.1</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
-        <v>-0.0343444398598879</v>
+        <v>0</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>2.81149719011719</v>
+        <v>2.78695615251733</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>3.53664746257987</v>
+        <v>3.47125014587866</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2.62916190926958</v>
+        <v>2.5857234814732</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.85990365566466</v>
+        <v>3.8125221071032</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0.37217140105922</v>
+        <v>0.48747591522158</v>
       </c>
       <c r="N7" s="14" t="n">
-        <v>0.14084492730938</v>
+        <v>0.153357722039176</v>
       </c>
       <c r="O7" s="15" t="n">
         <f aca="false">1-N7</f>
-        <v>0.85915507269062</v>
+        <v>0.846642277960824</v>
       </c>
       <c r="P7" s="13" t="n">
-        <v>0.271545498314877</v>
+        <v>0.293352601156069</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>0.810022026431718</v>
+        <v>0.821487603305785</v>
       </c>
       <c r="R7" s="13" t="n">
-        <v>0.841796875</v>
+        <v>0.827788649706458</v>
       </c>
       <c r="S7" s="16" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily oil & gas forecast 2026-10-27
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
@@ -432,34 +432,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -605,7 +605,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="G13:K23"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="8" style="0" width="13"/>
@@ -733,7 +733,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:S12"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="9"/>

</xml_diff>

<commit_message>
Daily oil & gas forecast 2026-10-29
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Henry Hub ($/MMBtu)</t>
   </si>
   <si>
-    <t xml:space="preserve">Forecast made on prices up to 2026-10-20; 7 day = 2026-10-27, 15 day = 2026-11-04.</t>
+    <t xml:space="preserve">Forecast made on prices up to 2026-10-27; 7 day = 2026-11-03, 15 day = 2026-11-11.</t>
   </si>
   <si>
     <t xml:space="preserve">Prices in $/bbl except Henry Hub ($/MMBtu).</t>
@@ -639,19 +639,19 @@
       </c>
       <c r="H16" s="5" t="n">
         <f aca="false">Details!G2</f>
-        <v>115.22</v>
+        <v>123.1</v>
       </c>
       <c r="I16" s="6" t="n">
         <f aca="false">Details!O2</f>
-        <v>0.953555293492327</v>
+        <v>0.953551045437089</v>
       </c>
       <c r="J16" s="5" t="n">
         <f aca="false">Details!G3</f>
-        <v>115.22</v>
+        <v>123.1</v>
       </c>
       <c r="K16" s="6" t="n">
         <f aca="false">Details!O3</f>
-        <v>0.931226967224115</v>
+        <v>0.931442443160265</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -660,19 +660,19 @@
       </c>
       <c r="H17" s="5" t="n">
         <f aca="false">Details!G4</f>
-        <v>107.89</v>
+        <v>103.37</v>
       </c>
       <c r="I17" s="6" t="n">
         <f aca="false">Details!O4</f>
-        <v>0.953872727483083</v>
+        <v>0.953874720659574</v>
       </c>
       <c r="J17" s="5" t="n">
         <f aca="false">Details!G5</f>
-        <v>107.89</v>
+        <v>103.37</v>
       </c>
       <c r="K17" s="6" t="n">
         <f aca="false">Details!O5</f>
-        <v>0.931561064272199</v>
+        <v>0.931620955590168</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -681,19 +681,19 @@
       </c>
       <c r="H18" s="5" t="n">
         <f aca="false">Details!G6</f>
-        <v>3.1</v>
+        <v>2.76</v>
       </c>
       <c r="I18" s="6" t="n">
         <f aca="false">Details!O6</f>
-        <v>0.890135513243169</v>
+        <v>0.889792455972064</v>
       </c>
       <c r="J18" s="5" t="n">
         <f aca="false">Details!G7</f>
-        <v>3.1</v>
+        <v>2.76</v>
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Details!O7</f>
-        <v>0.846642277960824</v>
+        <v>0.846576761223249</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -819,51 +819,51 @@
         <v>7</v>
       </c>
       <c r="D2" s="10" t="n">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="E2" s="10" t="n">
-        <v>46322</v>
+        <v>46329</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>115.22</v>
+        <v>123.1</v>
       </c>
       <c r="G2" s="11" t="n">
-        <v>115.22</v>
+        <v>123.1</v>
       </c>
       <c r="H2" s="12" t="n">
         <f aca="false">G2/F2-1</f>
         <v>0</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>101.308872623481</v>
+        <v>108.90360863425</v>
       </c>
       <c r="J2" s="11" t="n">
-        <v>130.171709702822</v>
+        <v>138.339007547121</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>91.6669081069355</v>
+        <v>99.253635145105</v>
       </c>
       <c r="L2" s="11" t="n">
-        <v>139.792901681923</v>
+        <v>148.104316503586</v>
       </c>
       <c r="M2" s="13" t="n">
-        <v>0.53314121037464</v>
+        <v>0.534582132564842</v>
       </c>
       <c r="N2" s="14" t="n">
-        <v>0.046444706507673</v>
+        <v>0.0464489545629107</v>
       </c>
       <c r="O2" s="15" t="n">
         <f aca="false">1-N2</f>
-        <v>0.953555293492327</v>
+        <v>0.953551045437089</v>
       </c>
       <c r="P2" s="13" t="n">
-        <v>0.69164265129683</v>
+        <v>0.690682036503362</v>
       </c>
       <c r="Q2" s="13" t="n">
-        <v>0.784345922276957</v>
+        <v>0.780514504652436</v>
       </c>
       <c r="R2" s="13" t="n">
-        <v>0.789168278529981</v>
+        <v>0.787234042553192</v>
       </c>
       <c r="S2" s="16" t="s">
         <v>31</v>
@@ -880,51 +880,51 @@
         <v>15</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>46330</v>
+        <v>46337</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>115.22</v>
+        <v>123.1</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>115.22</v>
+        <v>123.1</v>
       </c>
       <c r="H3" s="12" t="n">
         <f aca="false">G3/F3-1</f>
         <v>0</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>94.8479044038997</v>
+        <v>102.410397428633</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>138.17221400397</v>
+        <v>146.461453545136</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>80.7498111838232</v>
+        <v>88.7332343729111</v>
       </c>
       <c r="L3" s="11" t="n">
-        <v>157.766705422609</v>
+        <v>166.270704765676</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>0.553468208092486</v>
       </c>
       <c r="N3" s="14" t="n">
-        <v>0.0687730327758854</v>
+        <v>0.0685575568397347</v>
       </c>
       <c r="O3" s="15" t="n">
         <f aca="false">1-N3</f>
-        <v>0.931226967224115</v>
+        <v>0.931442443160265</v>
       </c>
       <c r="P3" s="13" t="n">
-        <v>0.533718689788054</v>
+        <v>0.535163776493256</v>
       </c>
       <c r="Q3" s="13" t="n">
-        <v>0.788980716253444</v>
+        <v>0.785123966942149</v>
       </c>
       <c r="R3" s="13" t="n">
-        <v>0.772994129158513</v>
+        <v>0.76908023483366</v>
       </c>
       <c r="S3" s="16" t="s">
         <v>31</v>
@@ -941,45 +941,45 @@
         <v>7</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>46322</v>
+        <v>46329</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>107.89</v>
+        <v>103.37</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>107.89</v>
+        <v>103.37</v>
       </c>
       <c r="H4" s="12" t="n">
         <f aca="false">G4/F4-1</f>
         <v>0</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>95.4250684796895</v>
+        <v>92.0121535996662</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>120.70865748815</v>
+        <v>115.068954323374</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>86.710635653351</v>
+        <v>83.8987749028762</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>128.081793069465</v>
+        <v>121.772354947906</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>0.538424591738713</v>
+        <v>0.539385206532181</v>
       </c>
       <c r="N4" s="14" t="n">
-        <v>0.0461272725169175</v>
+        <v>0.0461252793404265</v>
       </c>
       <c r="O4" s="15" t="n">
         <f aca="false">1-N4</f>
-        <v>0.953872727483083</v>
+        <v>0.953874720659574</v>
       </c>
       <c r="P4" s="13" t="n">
-        <v>0.698366954851105</v>
+        <v>0.698847262247839</v>
       </c>
       <c r="Q4" s="13" t="n">
         <v>0.799671592775041</v>
@@ -1002,51 +1002,51 @@
         <v>15</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>46330</v>
+        <v>46337</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>107.89</v>
+        <v>103.37</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>107.89</v>
+        <v>103.37</v>
       </c>
       <c r="H5" s="12" t="n">
         <f aca="false">G5/F5-1</f>
         <v>0</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>90.2883445378342</v>
+        <v>87.3385323784452</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>126.607148094806</v>
+        <v>120.433080071108</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>77.2523905273769</v>
+        <v>75.1366595942806</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>141.135917535299</v>
+        <v>133.598792042297</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>0.558285163776493</v>
+        <v>0.560693641618497</v>
       </c>
       <c r="N5" s="14" t="n">
-        <v>0.0684389357278012</v>
+        <v>0.0683790444098319</v>
       </c>
       <c r="O5" s="15" t="n">
         <f aca="false">1-N5</f>
-        <v>0.931561064272199</v>
+        <v>0.931620955590168</v>
       </c>
       <c r="P5" s="13" t="n">
         <v>0.536127167630058</v>
       </c>
       <c r="Q5" s="13" t="n">
-        <v>0.806060606060606</v>
+        <v>0.805509641873278</v>
       </c>
       <c r="R5" s="13" t="n">
-        <v>0.814090019569472</v>
+        <v>0.812133072407045</v>
       </c>
       <c r="S5" s="16" t="s">
         <v>31</v>
@@ -1063,51 +1063,51 @@
         <v>7</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>46322</v>
+        <v>46329</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>3.1</v>
+        <v>2.76</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>3.1</v>
+        <v>2.76</v>
       </c>
       <c r="H6" s="12" t="n">
         <f aca="false">G6/F6-1</f>
         <v>0</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>2.86517013121415</v>
+        <v>2.45852845604622</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>3.3598385873273</v>
+        <v>3.10326304702718</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>2.70824005693516</v>
+        <v>2.2583926097042</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>3.58831554209777</v>
+        <v>3.4153087281035</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>0.498559077809798</v>
       </c>
       <c r="N6" s="14" t="n">
-        <v>0.109864486756831</v>
+        <v>0.110207544027937</v>
       </c>
       <c r="O6" s="15" t="n">
         <f aca="false">1-N6</f>
-        <v>0.890135513243169</v>
+        <v>0.889792455972064</v>
       </c>
       <c r="P6" s="13" t="n">
-        <v>0.419308357348703</v>
+        <v>0.416906820365034</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>0.812807881773399</v>
+        <v>0.811165845648604</v>
       </c>
       <c r="R6" s="13" t="n">
-        <v>0.831721470019342</v>
+        <v>0.827852998065764</v>
       </c>
       <c r="S6" s="16" t="s">
         <v>31</v>
@@ -1124,48 +1124,48 @@
         <v>15</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>46330</v>
+        <v>46337</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>3.1</v>
+        <v>2.76</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>3.1</v>
+        <v>2.76</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
         <v>0</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>2.78695615251733</v>
+        <v>2.35605322743091</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>3.47125014587866</v>
+        <v>3.25191608878585</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2.5857234814732</v>
+        <v>2.11273376108439</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.8125221071032</v>
+        <v>3.71424054662121</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0.48747591522158</v>
+        <v>0.485067437379576</v>
       </c>
       <c r="N7" s="14" t="n">
-        <v>0.153357722039176</v>
+        <v>0.153423238776751</v>
       </c>
       <c r="O7" s="15" t="n">
         <f aca="false">1-N7</f>
-        <v>0.846642277960824</v>
+        <v>0.846576761223249</v>
       </c>
       <c r="P7" s="13" t="n">
         <v>0.293352601156069</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>0.821487603305785</v>
+        <v>0.82038567493113</v>
       </c>
       <c r="R7" s="13" t="n">
         <v>0.827788649706458</v>

</xml_diff>

<commit_message>
Daily oil & gas forecast 2026-10-31
</commit_message>
<xml_diff>
--- a/daily_forecasts/latest/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/latest/oil_gas_price_forecast.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="39">
   <si>
     <t xml:space="preserve">Crude oil Price forecast per bbl</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t xml:space="preserve">$/MMBtu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ridge + GBM ensemble</t>
   </si>
   <si>
     <t xml:space="preserve">Data: FRED / EIA APIs + EIA spot prices (github.com/datasets mirror). Blue = model output (python run_forecast.py); black = formula.</t>
@@ -689,11 +692,11 @@
       </c>
       <c r="J18" s="5" t="n">
         <f aca="false">Details!G7</f>
-        <v>2.76</v>
+        <v>2.76655965607836</v>
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Details!O7</f>
-        <v>0.846576761223249</v>
+        <v>0.858988414554952</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -972,7 +975,7 @@
         <v>0.539385206532181</v>
       </c>
       <c r="N4" s="14" t="n">
-        <v>0.0461252793404266</v>
+        <v>0.0461252793404265</v>
       </c>
       <c r="O4" s="15" t="n">
         <f aca="false">1-N4</f>
@@ -1133,65 +1136,65 @@
         <v>2.76</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>2.76</v>
+        <v>2.76655965607836</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
-        <v>0</v>
+        <v>0.00237668698491178</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>2.35605322743091</v>
+        <v>2.37843009572286</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>3.25191608878585</v>
+        <v>3.31432185426629</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2.11273376108439</v>
+        <v>2.14197258906726</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.71424054662121</v>
+        <v>3.77303586697696</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0.485067437379576</v>
+        <v>0.533718689788054</v>
       </c>
       <c r="N7" s="14" t="n">
-        <v>0.153423238776751</v>
+        <v>0.141011585445048</v>
       </c>
       <c r="O7" s="15" t="n">
         <f aca="false">1-N7</f>
-        <v>0.846576761223249</v>
+        <v>0.858988414554952</v>
       </c>
       <c r="P7" s="13" t="n">
-        <v>0.293352601156069</v>
+        <v>0.277938342967245</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>0.82038567493113</v>
+        <v>0.813774104683196</v>
       </c>
       <c r="R7" s="13" t="n">
-        <v>0.827788649706458</v>
+        <v>0.835616438356164</v>
       </c>
       <c r="S7" s="16" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>